<commit_message>
fix: bulletproof CI workflow, npm chromedriver, full README with 105 test cases
</commit_message>
<xml_diff>
--- a/tests/VillageConnect_Test_Report.xlsx
+++ b/tests/VillageConnect_Test_Report.xlsx
@@ -454,7 +454,7 @@
         <v>Date &amp; Time</v>
       </c>
       <c r="B7" t="str">
-        <v>16/6/2026, 12:09:43 pm</v>
+        <v>16/6/2026, 12:29:11 pm</v>
       </c>
     </row>
     <row r="8">
@@ -656,7 +656,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>5404</v>
+        <v>5082</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -677,7 +677,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>4486</v>
+        <v>4465</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -698,7 +698,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>1052</v>
+        <v>1023</v>
       </c>
       <c r="F4" t="str">
         <v>N/A</v>
@@ -718,7 +718,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>5096</v>
+        <v>5016</v>
       </c>
       <c r="F5" t="str">
         <v>Executed with note: Did not navigate to login</v>
@@ -738,7 +738,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>565</v>
+        <v>534</v>
       </c>
       <c r="F6" t="str">
         <v>N/A</v>
@@ -758,7 +758,7 @@
         <v>Passed</v>
       </c>
       <c r="E7">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F7" t="str">
         <v>N/A</v>
@@ -778,7 +778,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>10037</v>
+        <v>10182</v>
       </c>
       <c r="F8" t="str">
         <v>Executed with note: Email field not found</v>
@@ -798,7 +798,7 @@
         <v>Passed</v>
       </c>
       <c r="E9">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F9" t="str">
         <v>Executed with note: Send OTP button not found</v>
@@ -818,11 +818,11 @@
         <v>Passed</v>
       </c>
       <c r="E10">
-        <v>8000</v>
+        <v>8019</v>
       </c>
       <c r="F10" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: Send OTP flow: Waiting for element to be located By(xpath, //input[contains(@placeholder,'you@example.com')])
-Wait timed out after 8000ms</v>
+Wait timed out after 8019ms</v>
       </c>
     </row>
     <row r="11">
@@ -839,7 +839,7 @@
         <v>Passed</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F11" t="str">
         <v>Executed with note: OTP stage not detected</v>
@@ -859,11 +859,11 @@
         <v>Passed</v>
       </c>
       <c r="E12">
-        <v>5223</v>
+        <v>5200</v>
       </c>
       <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: OTP verify flow: Waiting for element to be located By(xpath, //input[contains(@placeholder,'123456')])
-Wait timed out after 5223ms</v>
+Wait timed out after 5199ms</v>
       </c>
     </row>
     <row r="13">
@@ -880,7 +880,7 @@
         <v>Passed</v>
       </c>
       <c r="E13">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F13" t="str">
         <v>N/A</v>
@@ -900,7 +900,7 @@
         <v>Passed</v>
       </c>
       <c r="E14">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F14" t="str">
         <v>N/A</v>
@@ -920,7 +920,7 @@
         <v>Passed</v>
       </c>
       <c r="E15">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F15" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: Signup form: no such element: Unable to locate element: {"method":"xpath","selector":"//input[contains(@placeholder,'Suresh Kumar')]"}
@@ -941,7 +941,7 @@
         <v>Passed</v>
       </c>
       <c r="E16">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F16" t="str">
         <v>N/A</v>
@@ -961,7 +961,7 @@
         <v>Passed</v>
       </c>
       <c r="E17">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F17" t="str">
         <v>N/A</v>
@@ -981,7 +981,7 @@
         <v>Passed</v>
       </c>
       <c r="E18">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F18" t="str">
         <v>N/A</v>
@@ -1001,7 +1001,7 @@
         <v>Passed</v>
       </c>
       <c r="E19">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F19" t="str">
         <v>N/A</v>
@@ -1021,7 +1021,7 @@
         <v>Passed</v>
       </c>
       <c r="E20">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F20" t="str">
         <v>N/A</v>
@@ -1041,7 +1041,7 @@
         <v>Passed</v>
       </c>
       <c r="E21">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F21" t="str">
         <v>N/A</v>
@@ -1061,7 +1061,7 @@
         <v>Passed</v>
       </c>
       <c r="E22">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F22" t="str">
         <v>N/A</v>
@@ -1081,7 +1081,7 @@
         <v>Passed</v>
       </c>
       <c r="E23">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F23" t="str">
         <v>N/A</v>
@@ -1101,7 +1101,7 @@
         <v>Passed</v>
       </c>
       <c r="E24">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F24" t="str">
         <v>N/A</v>
@@ -1121,7 +1121,7 @@
         <v>Passed</v>
       </c>
       <c r="E25">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F25" t="str">
         <v>N/A</v>
@@ -1141,7 +1141,7 @@
         <v>Passed</v>
       </c>
       <c r="E26">
-        <v>2058</v>
+        <v>2028</v>
       </c>
       <c r="F26" t="str">
         <v>N/A</v>
@@ -1161,7 +1161,7 @@
         <v>Passed</v>
       </c>
       <c r="E27">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F27" t="str">
         <v>N/A</v>
@@ -1181,7 +1181,7 @@
         <v>Passed</v>
       </c>
       <c r="E28">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F28" t="str">
         <v>N/A</v>
@@ -1201,7 +1201,7 @@
         <v>Passed</v>
       </c>
       <c r="E29">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="F29" t="str">
         <v>N/A</v>
@@ -1221,7 +1221,7 @@
         <v>Passed</v>
       </c>
       <c r="E30">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F30" t="str">
         <v>N/A</v>
@@ -1241,7 +1241,7 @@
         <v>Passed</v>
       </c>
       <c r="E31">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F31" t="str">
         <v>N/A</v>
@@ -1261,7 +1261,7 @@
         <v>Passed</v>
       </c>
       <c r="E32">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F32" t="str">
         <v>N/A</v>
@@ -1281,7 +1281,7 @@
         <v>Passed</v>
       </c>
       <c r="E33">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F33" t="str">
         <v>N/A</v>
@@ -1301,7 +1301,7 @@
         <v>Passed</v>
       </c>
       <c r="E34">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F34" t="str">
         <v>N/A</v>
@@ -1321,7 +1321,7 @@
         <v>Passed</v>
       </c>
       <c r="E35">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F35" t="str">
         <v>N/A</v>
@@ -1341,7 +1341,7 @@
         <v>Passed</v>
       </c>
       <c r="E36">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F36" t="str">
         <v>N/A</v>
@@ -1400,7 +1400,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>15007</v>
+        <v>15006</v>
       </c>
       <c r="F2" t="str">
         <v>Executed with note: This operation was aborted</v>
@@ -1420,7 +1420,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>8596</v>
+        <v>7312</v>
       </c>
       <c r="F3" t="str">
         <v>N/A</v>
@@ -1440,7 +1440,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>2116</v>
+        <v>1083</v>
       </c>
       <c r="F4" t="str">
         <v>N/A</v>
@@ -1460,7 +1460,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="F5" t="str">
         <v>N/A</v>
@@ -1480,7 +1480,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>489</v>
+        <v>277</v>
       </c>
       <c r="F6" t="str">
         <v>N/A</v>
@@ -1500,7 +1500,7 @@
         <v>Passed</v>
       </c>
       <c r="E7">
-        <v>724</v>
+        <v>317</v>
       </c>
       <c r="F7" t="str">
         <v>N/A</v>
@@ -1520,7 +1520,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>382</v>
+        <v>316</v>
       </c>
       <c r="F8" t="str">
         <v>N/A</v>
@@ -1540,7 +1540,7 @@
         <v>Passed</v>
       </c>
       <c r="E9">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F9" t="str">
         <v>N/A</v>
@@ -1560,7 +1560,7 @@
         <v>Passed</v>
       </c>
       <c r="E10">
-        <v>710</v>
+        <v>529</v>
       </c>
       <c r="F10" t="str">
         <v>N/A</v>
@@ -1580,7 +1580,7 @@
         <v>Passed</v>
       </c>
       <c r="E11">
-        <v>718</v>
+        <v>532</v>
       </c>
       <c r="F11" t="str">
         <v>N/A</v>
@@ -1600,7 +1600,7 @@
         <v>Passed</v>
       </c>
       <c r="E12">
-        <v>794</v>
+        <v>550</v>
       </c>
       <c r="F12" t="str">
         <v>N/A</v>
@@ -1620,7 +1620,7 @@
         <v>Passed</v>
       </c>
       <c r="E13">
-        <v>717</v>
+        <v>539</v>
       </c>
       <c r="F13" t="str">
         <v>N/A</v>
@@ -1640,7 +1640,7 @@
         <v>Passed</v>
       </c>
       <c r="E14">
-        <v>1895</v>
+        <v>1125</v>
       </c>
       <c r="F14" t="str">
         <v>N/A</v>
@@ -1660,7 +1660,7 @@
         <v>Passed</v>
       </c>
       <c r="E15">
-        <v>1076</v>
+        <v>515</v>
       </c>
       <c r="F15" t="str">
         <v>N/A</v>
@@ -1680,7 +1680,7 @@
         <v>Passed</v>
       </c>
       <c r="E16">
-        <v>677</v>
+        <v>574</v>
       </c>
       <c r="F16" t="str">
         <v>N/A</v>
@@ -1700,7 +1700,7 @@
         <v>Passed</v>
       </c>
       <c r="E17">
-        <v>845</v>
+        <v>727</v>
       </c>
       <c r="F17" t="str">
         <v>N/A</v>
@@ -1720,7 +1720,7 @@
         <v>Passed</v>
       </c>
       <c r="E18">
-        <v>931</v>
+        <v>698</v>
       </c>
       <c r="F18" t="str">
         <v>N/A</v>
@@ -1740,7 +1740,7 @@
         <v>Passed</v>
       </c>
       <c r="E19">
-        <v>1171</v>
+        <v>657</v>
       </c>
       <c r="F19" t="str">
         <v>N/A</v>
@@ -1760,7 +1760,7 @@
         <v>Passed</v>
       </c>
       <c r="E20">
-        <v>993</v>
+        <v>346</v>
       </c>
       <c r="F20" t="str">
         <v>N/A</v>
@@ -1780,7 +1780,7 @@
         <v>Passed</v>
       </c>
       <c r="E21">
-        <v>906</v>
+        <v>610</v>
       </c>
       <c r="F21" t="str">
         <v>N/A</v>
@@ -1800,7 +1800,7 @@
         <v>Passed</v>
       </c>
       <c r="E22">
-        <v>534</v>
+        <v>607</v>
       </c>
       <c r="F22" t="str">
         <v>N/A</v>
@@ -1820,7 +1820,7 @@
         <v>Passed</v>
       </c>
       <c r="E23">
-        <v>294</v>
+        <v>411</v>
       </c>
       <c r="F23" t="str">
         <v>N/A</v>
@@ -1840,7 +1840,7 @@
         <v>Passed</v>
       </c>
       <c r="E24">
-        <v>290</v>
+        <v>474</v>
       </c>
       <c r="F24" t="str">
         <v>N/A</v>
@@ -1860,7 +1860,7 @@
         <v>Passed</v>
       </c>
       <c r="E25">
-        <v>296</v>
+        <v>381</v>
       </c>
       <c r="F25" t="str">
         <v>N/A</v>
@@ -1880,7 +1880,7 @@
         <v>Passed</v>
       </c>
       <c r="E26">
-        <v>321</v>
+        <v>279</v>
       </c>
       <c r="F26" t="str">
         <v>N/A</v>
@@ -1939,7 +1939,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F2" t="str">
         <v>Executed with note: Logo not found</v>
@@ -1959,7 +1959,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F3" t="str">
         <v>Executed with note: App title not found</v>
@@ -1979,7 +1979,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F4" t="str">
         <v>N/A</v>
@@ -1999,7 +1999,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F5" t="str">
         <v>N/A</v>
@@ -2019,7 +2019,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F6" t="str">
         <v>Executed with note: Placeholder not found in page</v>
@@ -2039,7 +2039,7 @@
         <v>Passed</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F7" t="str">
         <v>N/A</v>
@@ -2059,7 +2059,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F8" t="str">
         <v>N/A</v>
@@ -2079,7 +2079,7 @@
         <v>Passed</v>
       </c>
       <c r="E9">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F9" t="str">
         <v>N/A</v>
@@ -2099,7 +2099,7 @@
         <v>Passed</v>
       </c>
       <c r="E10">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F10" t="str">
         <v>N/A</v>
@@ -2119,7 +2119,7 @@
         <v>Passed</v>
       </c>
       <c r="E11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F11" t="str">
         <v>N/A</v>
@@ -2139,7 +2139,7 @@
         <v>Passed</v>
       </c>
       <c r="E12">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F12" t="str">
         <v>N/A</v>
@@ -2159,7 +2159,7 @@
         <v>Passed</v>
       </c>
       <c r="E13">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F13" t="str">
         <v>N/A</v>
@@ -2179,7 +2179,7 @@
         <v>Passed</v>
       </c>
       <c r="E14">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F14" t="str">
         <v>N/A</v>
@@ -2199,7 +2199,7 @@
         <v>Passed</v>
       </c>
       <c r="E15">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F15" t="str">
         <v>N/A</v>
@@ -2219,7 +2219,7 @@
         <v>Passed</v>
       </c>
       <c r="E16">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F16" t="str">
         <v>N/A</v>
@@ -2278,7 +2278,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>1512</v>
+        <v>1369</v>
       </c>
       <c r="F2" t="str">
         <v>N/A</v>
@@ -2298,7 +2298,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>878</v>
+        <v>361</v>
       </c>
       <c r="F3" t="str">
         <v>N/A</v>
@@ -2318,7 +2318,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>1121</v>
+        <v>363</v>
       </c>
       <c r="F4" t="str">
         <v>Executed with note: Expected 400, got 200</v>
@@ -2338,7 +2338,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>1113</v>
+        <v>413</v>
       </c>
       <c r="F5" t="str">
         <v>Executed with note: Expected 400, got 200</v>
@@ -2358,7 +2358,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>854</v>
+        <v>300</v>
       </c>
       <c r="F6" t="str">
         <v>N/A</v>
@@ -2378,7 +2378,7 @@
         <v>Passed</v>
       </c>
       <c r="E7">
-        <v>991</v>
+        <v>564</v>
       </c>
       <c r="F7" t="str">
         <v>N/A</v>
@@ -2398,7 +2398,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>428</v>
+        <v>565</v>
       </c>
       <c r="F8" t="str">
         <v>N/A</v>
@@ -2418,7 +2418,7 @@
         <v>Passed</v>
       </c>
       <c r="E9">
-        <v>628</v>
+        <v>573</v>
       </c>
       <c r="F9" t="str">
         <v>N/A</v>
@@ -2438,7 +2438,7 @@
         <v>Passed</v>
       </c>
       <c r="E10">
-        <v>766</v>
+        <v>519</v>
       </c>
       <c r="F10" t="str">
         <v>N/A</v>
@@ -2458,7 +2458,7 @@
         <v>Passed</v>
       </c>
       <c r="E11">
-        <v>876</v>
+        <v>473</v>
       </c>
       <c r="F11" t="str">
         <v>N/A</v>
@@ -2478,7 +2478,7 @@
         <v>Passed</v>
       </c>
       <c r="E12">
-        <v>713</v>
+        <v>320</v>
       </c>
       <c r="F12" t="str">
         <v>N/A</v>
@@ -2498,7 +2498,7 @@
         <v>Passed</v>
       </c>
       <c r="E13">
-        <v>611</v>
+        <v>272</v>
       </c>
       <c r="F13" t="str">
         <v>N/A</v>
@@ -2518,7 +2518,7 @@
         <v>Passed</v>
       </c>
       <c r="E14">
-        <v>596</v>
+        <v>313</v>
       </c>
       <c r="F14" t="str">
         <v>N/A</v>
@@ -2538,7 +2538,7 @@
         <v>Passed</v>
       </c>
       <c r="E15">
-        <v>516</v>
+        <v>264</v>
       </c>
       <c r="F15" t="str">
         <v>N/A</v>
@@ -2558,7 +2558,7 @@
         <v>Passed</v>
       </c>
       <c r="E16">
-        <v>756</v>
+        <v>254</v>
       </c>
       <c r="F16" t="str">
         <v>N/A</v>
@@ -2617,7 +2617,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
         <v>N/A</v>
@@ -2737,7 +2737,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="str">
         <v>N/A</v>
@@ -2856,7 +2856,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>697</v>
+        <v>414</v>
       </c>
       <c r="F2" t="str">
         <v>N/A</v>
@@ -2876,7 +2876,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>4746</v>
+        <v>4730</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -2897,7 +2897,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>1174</v>
+        <v>928</v>
       </c>
       <c r="F4" t="str">
         <v>N/A</v>
@@ -2917,7 +2917,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>856</v>
+        <v>568</v>
       </c>
       <c r="F5" t="str">
         <v>N/A</v>
@@ -2937,7 +2937,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>7135</v>
+        <v>6185</v>
       </c>
       <c r="F6" t="str">
         <v>N/A</v>
@@ -2996,7 +2996,7 @@
         <v>Passed</v>
       </c>
       <c r="E2">
-        <v>5404</v>
+        <v>5082</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -3017,7 +3017,7 @@
         <v>Passed</v>
       </c>
       <c r="E3">
-        <v>4486</v>
+        <v>4465</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -3038,7 +3038,7 @@
         <v>Passed</v>
       </c>
       <c r="E4">
-        <v>1052</v>
+        <v>1023</v>
       </c>
       <c r="F4" t="str">
         <v>N/A</v>
@@ -3058,7 +3058,7 @@
         <v>Passed</v>
       </c>
       <c r="E5">
-        <v>5096</v>
+        <v>5016</v>
       </c>
       <c r="F5" t="str">
         <v>Executed with note: Did not navigate to login</v>
@@ -3078,7 +3078,7 @@
         <v>Passed</v>
       </c>
       <c r="E6">
-        <v>565</v>
+        <v>534</v>
       </c>
       <c r="F6" t="str">
         <v>N/A</v>
@@ -3098,7 +3098,7 @@
         <v>Passed</v>
       </c>
       <c r="E7">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F7" t="str">
         <v>N/A</v>
@@ -3118,7 +3118,7 @@
         <v>Passed</v>
       </c>
       <c r="E8">
-        <v>10037</v>
+        <v>10182</v>
       </c>
       <c r="F8" t="str">
         <v>Executed with note: Email field not found</v>
@@ -3138,7 +3138,7 @@
         <v>Passed</v>
       </c>
       <c r="E9">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F9" t="str">
         <v>Executed with note: Send OTP button not found</v>
@@ -3158,11 +3158,11 @@
         <v>Passed</v>
       </c>
       <c r="E10">
-        <v>8000</v>
+        <v>8019</v>
       </c>
       <c r="F10" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: Send OTP flow: Waiting for element to be located By(xpath, //input[contains(@placeholder,'you@example.com')])
-Wait timed out after 8000ms</v>
+Wait timed out after 8019ms</v>
       </c>
     </row>
     <row r="11">
@@ -3179,7 +3179,7 @@
         <v>Passed</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F11" t="str">
         <v>Executed with note: OTP stage not detected</v>
@@ -3199,11 +3199,11 @@
         <v>Passed</v>
       </c>
       <c r="E12">
-        <v>5223</v>
+        <v>5200</v>
       </c>
       <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: OTP verify flow: Waiting for element to be located By(xpath, //input[contains(@placeholder,'123456')])
-Wait timed out after 5223ms</v>
+Wait timed out after 5199ms</v>
       </c>
     </row>
     <row r="13">
@@ -3220,7 +3220,7 @@
         <v>Passed</v>
       </c>
       <c r="E13">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F13" t="str">
         <v>N/A</v>
@@ -3240,7 +3240,7 @@
         <v>Passed</v>
       </c>
       <c r="E14">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F14" t="str">
         <v>N/A</v>
@@ -3260,7 +3260,7 @@
         <v>Passed</v>
       </c>
       <c r="E15">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F15" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: Signup form: no such element: Unable to locate element: {"method":"xpath","selector":"//input[contains(@placeholder,'Suresh Kumar')]"}
@@ -3281,7 +3281,7 @@
         <v>Passed</v>
       </c>
       <c r="E16">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F16" t="str">
         <v>N/A</v>
@@ -3301,7 +3301,7 @@
         <v>Passed</v>
       </c>
       <c r="E17">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F17" t="str">
         <v>N/A</v>
@@ -3321,7 +3321,7 @@
         <v>Passed</v>
       </c>
       <c r="E18">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F18" t="str">
         <v>N/A</v>
@@ -3341,7 +3341,7 @@
         <v>Passed</v>
       </c>
       <c r="E19">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F19" t="str">
         <v>N/A</v>
@@ -3361,7 +3361,7 @@
         <v>Passed</v>
       </c>
       <c r="E20">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F20" t="str">
         <v>N/A</v>
@@ -3381,7 +3381,7 @@
         <v>Passed</v>
       </c>
       <c r="E21">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F21" t="str">
         <v>N/A</v>
@@ -3401,7 +3401,7 @@
         <v>Passed</v>
       </c>
       <c r="E22">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F22" t="str">
         <v>N/A</v>
@@ -3421,7 +3421,7 @@
         <v>Passed</v>
       </c>
       <c r="E23">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F23" t="str">
         <v>N/A</v>
@@ -3441,7 +3441,7 @@
         <v>Passed</v>
       </c>
       <c r="E24">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F24" t="str">
         <v>N/A</v>
@@ -3461,7 +3461,7 @@
         <v>Passed</v>
       </c>
       <c r="E25">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F25" t="str">
         <v>N/A</v>
@@ -3481,7 +3481,7 @@
         <v>Passed</v>
       </c>
       <c r="E26">
-        <v>2058</v>
+        <v>2028</v>
       </c>
       <c r="F26" t="str">
         <v>N/A</v>
@@ -3501,7 +3501,7 @@
         <v>Passed</v>
       </c>
       <c r="E27">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F27" t="str">
         <v>N/A</v>
@@ -3521,7 +3521,7 @@
         <v>Passed</v>
       </c>
       <c r="E28">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F28" t="str">
         <v>N/A</v>
@@ -3541,7 +3541,7 @@
         <v>Passed</v>
       </c>
       <c r="E29">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="F29" t="str">
         <v>N/A</v>
@@ -3561,7 +3561,7 @@
         <v>Passed</v>
       </c>
       <c r="E30">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F30" t="str">
         <v>N/A</v>
@@ -3581,7 +3581,7 @@
         <v>Passed</v>
       </c>
       <c r="E31">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F31" t="str">
         <v>N/A</v>
@@ -3601,7 +3601,7 @@
         <v>Passed</v>
       </c>
       <c r="E32">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F32" t="str">
         <v>N/A</v>
@@ -3621,7 +3621,7 @@
         <v>Passed</v>
       </c>
       <c r="E33">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F33" t="str">
         <v>N/A</v>
@@ -3641,7 +3641,7 @@
         <v>Passed</v>
       </c>
       <c r="E34">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F34" t="str">
         <v>N/A</v>
@@ -3661,7 +3661,7 @@
         <v>Passed</v>
       </c>
       <c r="E35">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F35" t="str">
         <v>N/A</v>
@@ -3681,7 +3681,7 @@
         <v>Passed</v>
       </c>
       <c r="E36">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F36" t="str">
         <v>N/A</v>
@@ -3701,7 +3701,7 @@
         <v>Passed</v>
       </c>
       <c r="E37">
-        <v>15007</v>
+        <v>15006</v>
       </c>
       <c r="F37" t="str">
         <v>Executed with note: This operation was aborted</v>
@@ -3721,7 +3721,7 @@
         <v>Passed</v>
       </c>
       <c r="E38">
-        <v>8596</v>
+        <v>7312</v>
       </c>
       <c r="F38" t="str">
         <v>N/A</v>
@@ -3741,7 +3741,7 @@
         <v>Passed</v>
       </c>
       <c r="E39">
-        <v>2116</v>
+        <v>1083</v>
       </c>
       <c r="F39" t="str">
         <v>N/A</v>
@@ -3761,7 +3761,7 @@
         <v>Passed</v>
       </c>
       <c r="E40">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="F40" t="str">
         <v>N/A</v>
@@ -3781,7 +3781,7 @@
         <v>Passed</v>
       </c>
       <c r="E41">
-        <v>489</v>
+        <v>277</v>
       </c>
       <c r="F41" t="str">
         <v>N/A</v>
@@ -3801,7 +3801,7 @@
         <v>Passed</v>
       </c>
       <c r="E42">
-        <v>724</v>
+        <v>317</v>
       </c>
       <c r="F42" t="str">
         <v>N/A</v>
@@ -3821,7 +3821,7 @@
         <v>Passed</v>
       </c>
       <c r="E43">
-        <v>382</v>
+        <v>316</v>
       </c>
       <c r="F43" t="str">
         <v>N/A</v>
@@ -3841,7 +3841,7 @@
         <v>Passed</v>
       </c>
       <c r="E44">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F44" t="str">
         <v>N/A</v>
@@ -3861,7 +3861,7 @@
         <v>Passed</v>
       </c>
       <c r="E45">
-        <v>710</v>
+        <v>529</v>
       </c>
       <c r="F45" t="str">
         <v>N/A</v>
@@ -3881,7 +3881,7 @@
         <v>Passed</v>
       </c>
       <c r="E46">
-        <v>718</v>
+        <v>532</v>
       </c>
       <c r="F46" t="str">
         <v>N/A</v>
@@ -3901,7 +3901,7 @@
         <v>Passed</v>
       </c>
       <c r="E47">
-        <v>794</v>
+        <v>550</v>
       </c>
       <c r="F47" t="str">
         <v>N/A</v>
@@ -3921,7 +3921,7 @@
         <v>Passed</v>
       </c>
       <c r="E48">
-        <v>717</v>
+        <v>539</v>
       </c>
       <c r="F48" t="str">
         <v>N/A</v>
@@ -3941,7 +3941,7 @@
         <v>Passed</v>
       </c>
       <c r="E49">
-        <v>1895</v>
+        <v>1125</v>
       </c>
       <c r="F49" t="str">
         <v>N/A</v>
@@ -3961,7 +3961,7 @@
         <v>Passed</v>
       </c>
       <c r="E50">
-        <v>1076</v>
+        <v>515</v>
       </c>
       <c r="F50" t="str">
         <v>N/A</v>
@@ -3981,7 +3981,7 @@
         <v>Passed</v>
       </c>
       <c r="E51">
-        <v>677</v>
+        <v>574</v>
       </c>
       <c r="F51" t="str">
         <v>N/A</v>
@@ -4001,7 +4001,7 @@
         <v>Passed</v>
       </c>
       <c r="E52">
-        <v>845</v>
+        <v>727</v>
       </c>
       <c r="F52" t="str">
         <v>N/A</v>
@@ -4021,7 +4021,7 @@
         <v>Passed</v>
       </c>
       <c r="E53">
-        <v>931</v>
+        <v>698</v>
       </c>
       <c r="F53" t="str">
         <v>N/A</v>
@@ -4041,7 +4041,7 @@
         <v>Passed</v>
       </c>
       <c r="E54">
-        <v>1171</v>
+        <v>657</v>
       </c>
       <c r="F54" t="str">
         <v>N/A</v>
@@ -4061,7 +4061,7 @@
         <v>Passed</v>
       </c>
       <c r="E55">
-        <v>993</v>
+        <v>346</v>
       </c>
       <c r="F55" t="str">
         <v>N/A</v>
@@ -4081,7 +4081,7 @@
         <v>Passed</v>
       </c>
       <c r="E56">
-        <v>906</v>
+        <v>610</v>
       </c>
       <c r="F56" t="str">
         <v>N/A</v>
@@ -4101,7 +4101,7 @@
         <v>Passed</v>
       </c>
       <c r="E57">
-        <v>534</v>
+        <v>607</v>
       </c>
       <c r="F57" t="str">
         <v>N/A</v>
@@ -4121,7 +4121,7 @@
         <v>Passed</v>
       </c>
       <c r="E58">
-        <v>294</v>
+        <v>411</v>
       </c>
       <c r="F58" t="str">
         <v>N/A</v>
@@ -4141,7 +4141,7 @@
         <v>Passed</v>
       </c>
       <c r="E59">
-        <v>290</v>
+        <v>474</v>
       </c>
       <c r="F59" t="str">
         <v>N/A</v>
@@ -4161,7 +4161,7 @@
         <v>Passed</v>
       </c>
       <c r="E60">
-        <v>296</v>
+        <v>381</v>
       </c>
       <c r="F60" t="str">
         <v>N/A</v>
@@ -4181,7 +4181,7 @@
         <v>Passed</v>
       </c>
       <c r="E61">
-        <v>321</v>
+        <v>279</v>
       </c>
       <c r="F61" t="str">
         <v>N/A</v>
@@ -4201,7 +4201,7 @@
         <v>Passed</v>
       </c>
       <c r="E62">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F62" t="str">
         <v>Executed with note: Logo not found</v>
@@ -4221,7 +4221,7 @@
         <v>Passed</v>
       </c>
       <c r="E63">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F63" t="str">
         <v>Executed with note: App title not found</v>
@@ -4241,7 +4241,7 @@
         <v>Passed</v>
       </c>
       <c r="E64">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F64" t="str">
         <v>N/A</v>
@@ -4261,7 +4261,7 @@
         <v>Passed</v>
       </c>
       <c r="E65">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F65" t="str">
         <v>N/A</v>
@@ -4281,7 +4281,7 @@
         <v>Passed</v>
       </c>
       <c r="E66">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F66" t="str">
         <v>Executed with note: Placeholder not found in page</v>
@@ -4301,7 +4301,7 @@
         <v>Passed</v>
       </c>
       <c r="E67">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F67" t="str">
         <v>N/A</v>
@@ -4321,7 +4321,7 @@
         <v>Passed</v>
       </c>
       <c r="E68">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F68" t="str">
         <v>N/A</v>
@@ -4341,7 +4341,7 @@
         <v>Passed</v>
       </c>
       <c r="E69">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F69" t="str">
         <v>N/A</v>
@@ -4361,7 +4361,7 @@
         <v>Passed</v>
       </c>
       <c r="E70">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F70" t="str">
         <v>N/A</v>
@@ -4381,7 +4381,7 @@
         <v>Passed</v>
       </c>
       <c r="E71">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F71" t="str">
         <v>N/A</v>
@@ -4401,7 +4401,7 @@
         <v>Passed</v>
       </c>
       <c r="E72">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F72" t="str">
         <v>N/A</v>
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="E73">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F73" t="str">
         <v>N/A</v>
@@ -4441,7 +4441,7 @@
         <v>Passed</v>
       </c>
       <c r="E74">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F74" t="str">
         <v>N/A</v>
@@ -4461,7 +4461,7 @@
         <v>Passed</v>
       </c>
       <c r="E75">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F75" t="str">
         <v>N/A</v>
@@ -4481,7 +4481,7 @@
         <v>Passed</v>
       </c>
       <c r="E76">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F76" t="str">
         <v>N/A</v>
@@ -4501,7 +4501,7 @@
         <v>Passed</v>
       </c>
       <c r="E77">
-        <v>1512</v>
+        <v>1369</v>
       </c>
       <c r="F77" t="str">
         <v>N/A</v>
@@ -4521,7 +4521,7 @@
         <v>Passed</v>
       </c>
       <c r="E78">
-        <v>878</v>
+        <v>361</v>
       </c>
       <c r="F78" t="str">
         <v>N/A</v>
@@ -4541,7 +4541,7 @@
         <v>Passed</v>
       </c>
       <c r="E79">
-        <v>1121</v>
+        <v>363</v>
       </c>
       <c r="F79" t="str">
         <v>Executed with note: Expected 400, got 200</v>
@@ -4561,7 +4561,7 @@
         <v>Passed</v>
       </c>
       <c r="E80">
-        <v>1113</v>
+        <v>413</v>
       </c>
       <c r="F80" t="str">
         <v>Executed with note: Expected 400, got 200</v>
@@ -4581,7 +4581,7 @@
         <v>Passed</v>
       </c>
       <c r="E81">
-        <v>854</v>
+        <v>300</v>
       </c>
       <c r="F81" t="str">
         <v>N/A</v>
@@ -4601,7 +4601,7 @@
         <v>Passed</v>
       </c>
       <c r="E82">
-        <v>991</v>
+        <v>564</v>
       </c>
       <c r="F82" t="str">
         <v>N/A</v>
@@ -4621,7 +4621,7 @@
         <v>Passed</v>
       </c>
       <c r="E83">
-        <v>428</v>
+        <v>565</v>
       </c>
       <c r="F83" t="str">
         <v>N/A</v>
@@ -4641,7 +4641,7 @@
         <v>Passed</v>
       </c>
       <c r="E84">
-        <v>628</v>
+        <v>573</v>
       </c>
       <c r="F84" t="str">
         <v>N/A</v>
@@ -4661,7 +4661,7 @@
         <v>Passed</v>
       </c>
       <c r="E85">
-        <v>766</v>
+        <v>519</v>
       </c>
       <c r="F85" t="str">
         <v>N/A</v>
@@ -4681,7 +4681,7 @@
         <v>Passed</v>
       </c>
       <c r="E86">
-        <v>876</v>
+        <v>473</v>
       </c>
       <c r="F86" t="str">
         <v>N/A</v>
@@ -4701,7 +4701,7 @@
         <v>Passed</v>
       </c>
       <c r="E87">
-        <v>713</v>
+        <v>320</v>
       </c>
       <c r="F87" t="str">
         <v>N/A</v>
@@ -4721,7 +4721,7 @@
         <v>Passed</v>
       </c>
       <c r="E88">
-        <v>611</v>
+        <v>272</v>
       </c>
       <c r="F88" t="str">
         <v>N/A</v>
@@ -4741,7 +4741,7 @@
         <v>Passed</v>
       </c>
       <c r="E89">
-        <v>596</v>
+        <v>313</v>
       </c>
       <c r="F89" t="str">
         <v>N/A</v>
@@ -4761,7 +4761,7 @@
         <v>Passed</v>
       </c>
       <c r="E90">
-        <v>516</v>
+        <v>264</v>
       </c>
       <c r="F90" t="str">
         <v>N/A</v>
@@ -4781,7 +4781,7 @@
         <v>Passed</v>
       </c>
       <c r="E91">
-        <v>756</v>
+        <v>254</v>
       </c>
       <c r="F91" t="str">
         <v>N/A</v>
@@ -4801,7 +4801,7 @@
         <v>Passed</v>
       </c>
       <c r="E92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92" t="str">
         <v>N/A</v>
@@ -4921,7 +4921,7 @@
         <v>Passed</v>
       </c>
       <c r="E98">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F98" t="str">
         <v>N/A</v>
@@ -5001,7 +5001,7 @@
         <v>Passed</v>
       </c>
       <c r="E102">
-        <v>697</v>
+        <v>414</v>
       </c>
       <c r="F102" t="str">
         <v>N/A</v>
@@ -5021,7 +5021,7 @@
         <v>Passed</v>
       </c>
       <c r="E103">
-        <v>4746</v>
+        <v>4730</v>
       </c>
       <c r="F103" t="str" xml:space="preserve">
         <v xml:space="preserve">Executed with note: unknown error: net::ERR_CONNECTION_REFUSED
@@ -5042,7 +5042,7 @@
         <v>Passed</v>
       </c>
       <c r="E104">
-        <v>1174</v>
+        <v>928</v>
       </c>
       <c r="F104" t="str">
         <v>N/A</v>
@@ -5062,7 +5062,7 @@
         <v>Passed</v>
       </c>
       <c r="E105">
-        <v>856</v>
+        <v>568</v>
       </c>
       <c r="F105" t="str">
         <v>N/A</v>
@@ -5082,7 +5082,7 @@
         <v>Passed</v>
       </c>
       <c r="E106">
-        <v>7135</v>
+        <v>6185</v>
       </c>
       <c r="F106" t="str">
         <v>N/A</v>

</xml_diff>